<commit_message>
chore(tasks): update implementation status
</commit_message>
<xml_diff>
--- a/Tasks.xlsx
+++ b/Tasks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jacopodonati/Documents/PROGETTI/TRAVELMINDER/ai-travel-planner/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/exler/VSCode_Projects/ai-travel-planner/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC8C1117-651F-C448-AF2C-887FE43AEF47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B20BBC4A-8766-3447-B355-51CB2FE6F212}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="33600" windowHeight="18860" xr2:uid="{834F46D4-8CFA-4605-9F2C-653FA769D6F4}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="33600" windowHeight="18860" xr2:uid="{834F46D4-8CFA-4605-9F2C-653FA769D6F4}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="204">
   <si>
     <t>Project Setup</t>
   </si>
@@ -844,7 +844,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -862,7 +862,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="de-DE"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1081,7 +1081,7 @@
                   <c:v>137</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>104</c:v>
+                  <c:v>99</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1984,7 +1984,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -2383,7 +2383,7 @@
         <v>0</v>
       </c>
       <c r="J5">
-        <f>COUNTIF($F$5:$F$199,H5)</f>
+        <f t="shared" ref="J5:J10" si="0">COUNTIF($F$5:$F$199,H5)</f>
         <v>0</v>
       </c>
       <c r="K5">
@@ -2417,7 +2417,7 @@
         <v>33</v>
       </c>
       <c r="J6">
-        <f>COUNTIF($F$5:$F$199,H6)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="K6">
@@ -2449,24 +2449,24 @@
         <v>2</v>
       </c>
       <c r="I7">
-        <f t="shared" ref="I7:I10" si="0">COUNTIF($B$5:$B$1900,H7)</f>
+        <f t="shared" ref="I7:I10" si="1">COUNTIF($B$5:$B$1900,H7)</f>
         <v>33</v>
       </c>
       <c r="J7">
-        <f>COUNTIF($F$5:$F$199,H7)</f>
-        <v>33</v>
+        <f t="shared" si="0"/>
+        <v>38</v>
       </c>
       <c r="K7">
-        <f t="shared" ref="K7:K10" si="1">K6-I7</f>
+        <f t="shared" ref="K7:K10" si="2">K6-I7</f>
         <v>99</v>
       </c>
       <c r="L7">
-        <f t="shared" ref="L7:L10" si="2">IF(H7&gt;$L$3,"",L6-J7)</f>
-        <v>104</v>
+        <f t="shared" ref="L7:L10" si="3">IF(H7&gt;$L$3,"",L6-J7)</f>
+        <v>99</v>
       </c>
       <c r="M7">
         <f>IF(H7&gt;$L$3,"",L7)</f>
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.2">
@@ -2489,19 +2489,19 @@
         <v>3</v>
       </c>
       <c r="I8">
+        <f t="shared" si="1"/>
+        <v>33</v>
+      </c>
+      <c r="J8">
         <f t="shared" si="0"/>
-        <v>33</v>
-      </c>
-      <c r="J8">
-        <f>COUNTIF($F$5:$F$199,H8)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="K8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>66</v>
       </c>
       <c r="L8" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="M8" t="str">
@@ -2529,19 +2529,19 @@
         <v>4</v>
       </c>
       <c r="I9">
+        <f t="shared" si="1"/>
+        <v>38</v>
+      </c>
+      <c r="J9">
         <f t="shared" si="0"/>
-        <v>38</v>
-      </c>
-      <c r="J9">
-        <f>COUNTIF($F$5:$F$199,H9)</f>
         <v>0</v>
       </c>
       <c r="K9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="L9" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="M9" t="str">
@@ -2569,19 +2569,19 @@
         <v>5</v>
       </c>
       <c r="I10">
+        <f t="shared" si="1"/>
+        <v>28</v>
+      </c>
+      <c r="J10">
         <f t="shared" si="0"/>
-        <v>28</v>
-      </c>
-      <c r="J10">
-        <f>COUNTIF($F$5:$F$199,H10)</f>
         <v>0</v>
       </c>
       <c r="K10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="L10" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="M10" t="str">
@@ -2983,6 +2983,9 @@
       <c r="E36" s="2" t="s">
         <v>29</v>
       </c>
+      <c r="F36">
+        <v>2</v>
+      </c>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B37">
@@ -2997,6 +3000,9 @@
       <c r="E37" s="2" t="s">
         <v>30</v>
       </c>
+      <c r="F37">
+        <v>2</v>
+      </c>
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B38">
@@ -3011,6 +3017,9 @@
       <c r="E38" s="2" t="s">
         <v>31</v>
       </c>
+      <c r="F38">
+        <v>2</v>
+      </c>
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B39">
@@ -3025,6 +3034,9 @@
       <c r="E39" s="2" t="s">
         <v>32</v>
       </c>
+      <c r="F39">
+        <v>2</v>
+      </c>
     </row>
     <row r="40" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B40">
@@ -3039,6 +3051,9 @@
       <c r="E40" s="2" t="s">
         <v>33</v>
       </c>
+      <c r="F40">
+        <v>2</v>
+      </c>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B42">
@@ -3605,16 +3620,25 @@
       <c r="B80">
         <v>3</v>
       </c>
+      <c r="C80" t="s">
+        <v>201</v>
+      </c>
       <c r="D80" s="3" t="s">
         <v>70</v>
       </c>
       <c r="E80" s="2" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="81" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F80">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="81" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B81">
         <v>3</v>
+      </c>
+      <c r="C81" t="s">
+        <v>201</v>
       </c>
       <c r="D81" s="3" t="s">
         <v>70</v>
@@ -3622,10 +3646,16 @@
       <c r="E81" s="2" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="82" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F81">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="82" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B82">
         <v>3</v>
+      </c>
+      <c r="C82" t="s">
+        <v>201</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>70</v>
@@ -3633,10 +3663,16 @@
       <c r="E82" s="2" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="83" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F82">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="83" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B83">
         <v>3</v>
+      </c>
+      <c r="C83" t="s">
+        <v>201</v>
       </c>
       <c r="D83" s="3" t="s">
         <v>70</v>
@@ -3644,10 +3680,16 @@
       <c r="E83" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="85" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F83">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="85" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B85">
         <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>201</v>
       </c>
       <c r="D85" s="3" t="s">
         <v>75</v>
@@ -3655,10 +3697,16 @@
       <c r="E85" s="2" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="86" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F85">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="86" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B86">
         <v>3</v>
+      </c>
+      <c r="C86" t="s">
+        <v>201</v>
       </c>
       <c r="D86" s="3" t="s">
         <v>75</v>
@@ -3666,10 +3714,16 @@
       <c r="E86" s="2" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="87" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F86">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="87" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B87">
         <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>201</v>
       </c>
       <c r="D87" s="3" t="s">
         <v>75</v>
@@ -3677,10 +3731,16 @@
       <c r="E87" s="2" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="88" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F87">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="88" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B88">
         <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>201</v>
       </c>
       <c r="D88" s="3" t="s">
         <v>75</v>
@@ -3688,10 +3748,16 @@
       <c r="E88" s="2" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="89" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F88">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="89" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B89">
         <v>3</v>
+      </c>
+      <c r="C89" t="s">
+        <v>201</v>
       </c>
       <c r="D89" s="3" t="s">
         <v>75</v>
@@ -3699,10 +3765,16 @@
       <c r="E89" s="2" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="90" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F89">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="90" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B90">
         <v>3</v>
+      </c>
+      <c r="C90" t="s">
+        <v>201</v>
       </c>
       <c r="D90" s="3" t="s">
         <v>75</v>
@@ -3710,10 +3782,16 @@
       <c r="E90" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="91" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F90">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="91" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B91">
         <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>201</v>
       </c>
       <c r="D91" s="3" t="s">
         <v>75</v>
@@ -3721,10 +3799,16 @@
       <c r="E91" s="2" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="92" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F91">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="92" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B92">
         <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>201</v>
       </c>
       <c r="D92" s="3" t="s">
         <v>75</v>
@@ -3732,10 +3816,16 @@
       <c r="E92" s="2" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="93" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F92">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="93" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B93">
         <v>3</v>
+      </c>
+      <c r="C93" t="s">
+        <v>201</v>
       </c>
       <c r="D93" s="3" t="s">
         <v>75</v>
@@ -3743,10 +3833,16 @@
       <c r="E93" s="2" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="94" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F93">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="94" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B94">
         <v>3</v>
+      </c>
+      <c r="C94" t="s">
+        <v>201</v>
       </c>
       <c r="D94" s="3" t="s">
         <v>75</v>
@@ -3754,16 +3850,25 @@
       <c r="E94" s="2" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="95" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F94">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="95" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B95">
         <v>3</v>
+      </c>
+      <c r="C95" t="s">
+        <v>201</v>
       </c>
       <c r="D95" s="3" t="s">
         <v>75</v>
       </c>
       <c r="E95" s="2" t="s">
         <v>86</v>
+      </c>
+      <c r="F95">
+        <v>3</v>
       </c>
     </row>
     <row r="97" spans="2:5" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
chore: update tasks spreadsheet
</commit_message>
<xml_diff>
--- a/Tasks.xlsx
+++ b/Tasks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pas02\Nextcloud\Documents\03_Data Science - Uni Stuttgart\06_SoS 2026\04_Software Engineering\Group project 3\ai-travel-planner\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jacopodonati/Documents/PROGETTI/TRAVELMINDER/ai-travel-planner/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B20BBC4A-8766-3447-B355-51CB2FE6F212}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6465E58-F374-294C-99D3-0E516C95C3C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="2940" windowWidth="21600" windowHeight="11295" xr2:uid="{834F46D4-8CFA-4605-9F2C-653FA769D6F4}"/>
+    <workbookView xWindow="2940" yWindow="2940" windowWidth="30440" windowHeight="16320" xr2:uid="{834F46D4-8CFA-4605-9F2C-653FA769D6F4}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="204">
   <si>
     <t>Project Setup</t>
   </si>
@@ -763,7 +763,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -844,7 +844,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -862,7 +862,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="de-DE"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1984,7 +1984,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -2301,16 +2301,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67F1D602-D536-4BC9-865A-CD2C06CAE9C2}">
   <dimension ref="B2:M193"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="6.85546875" customWidth="1"/>
-    <col min="3" max="3" width="22.85546875" customWidth="1"/>
-    <col min="4" max="4" width="29.7109375" customWidth="1"/>
-    <col min="5" max="5" width="66.140625" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="2" max="2" width="6.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="29.6640625" customWidth="1"/>
+    <col min="5" max="5" width="66.1640625" customWidth="1"/>
+    <col min="6" max="6" width="12.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" ht="21">
+    <row r="2" spans="2:13" ht="22" x14ac:dyDescent="0.3">
       <c r="B2" s="5" t="s">
         <v>191</v>
       </c>
@@ -2319,7 +2319,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="3" spans="2:13">
+    <row r="3" spans="2:13" x14ac:dyDescent="0.2">
       <c r="E3" s="4"/>
       <c r="K3" t="s">
         <v>199</v>
@@ -2328,7 +2328,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="2:13">
+    <row r="4" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
         <v>188</v>
       </c>
@@ -2360,7 +2360,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="5" spans="2:13">
+    <row r="5" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B5">
         <v>1</v>
       </c>
@@ -2393,7 +2393,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="6" spans="2:13">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B6">
         <v>1</v>
       </c>
@@ -2429,7 +2429,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="7" spans="2:13">
+    <row r="7" spans="2:13" ht="17" x14ac:dyDescent="0.2">
       <c r="B7">
         <v>1</v>
       </c>
@@ -2469,7 +2469,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="2:13">
+    <row r="8" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B8">
         <v>1</v>
       </c>
@@ -2494,7 +2494,7 @@
       </c>
       <c r="J8">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="K8">
         <f t="shared" si="2"/>
@@ -2509,7 +2509,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="2:13">
+    <row r="9" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B9">
         <v>1</v>
       </c>
@@ -2549,7 +2549,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="2:13">
+    <row r="10" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B10">
         <v>1</v>
       </c>
@@ -2589,7 +2589,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="2:13">
+    <row r="11" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B11">
         <v>1</v>
       </c>
@@ -2613,7 +2613,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="12" spans="2:13">
+    <row r="12" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B12">
         <v>1</v>
       </c>
@@ -2630,7 +2630,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="2:13">
+    <row r="14" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B14">
         <v>1</v>
       </c>
@@ -2647,7 +2647,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="2:13">
+    <row r="15" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B15">
         <v>1</v>
       </c>
@@ -2664,7 +2664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="2:13">
+    <row r="16" spans="2:13" ht="17" x14ac:dyDescent="0.2">
       <c r="B16">
         <v>1</v>
       </c>
@@ -2681,7 +2681,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:6">
+    <row r="17" spans="2:6" ht="17" x14ac:dyDescent="0.2">
       <c r="B17">
         <v>1</v>
       </c>
@@ -2698,7 +2698,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="2:6">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B18">
         <v>1</v>
       </c>
@@ -2715,7 +2715,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:6">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B19">
         <v>1</v>
       </c>
@@ -2732,7 +2732,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="2:6">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B20">
         <v>1</v>
       </c>
@@ -2749,7 +2749,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:6">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B22">
         <v>1</v>
       </c>
@@ -2766,7 +2766,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="2:6">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B23">
         <v>1</v>
       </c>
@@ -2783,7 +2783,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="2:6">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B24">
         <v>1</v>
       </c>
@@ -2800,7 +2800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="2:6">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B25">
         <v>1</v>
       </c>
@@ -2817,7 +2817,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="2:6">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B26">
         <v>1</v>
       </c>
@@ -2834,7 +2834,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="2:6">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B27">
         <v>1</v>
       </c>
@@ -2851,7 +2851,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="2:6">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B28">
         <v>1</v>
       </c>
@@ -2868,7 +2868,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:6">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B29">
         <v>1</v>
       </c>
@@ -2885,7 +2885,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="2:6">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B30">
         <v>1</v>
       </c>
@@ -2902,7 +2902,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="2:6">
+    <row r="31" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B31">
         <v>1</v>
       </c>
@@ -2919,7 +2919,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="2:6">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B32">
         <v>1</v>
       </c>
@@ -2936,7 +2936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="2:6">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B33">
         <v>1</v>
       </c>
@@ -2953,7 +2953,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="2:6">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B34">
         <v>1</v>
       </c>
@@ -2970,7 +2970,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="2:6">
+    <row r="36" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B36">
         <v>1</v>
       </c>
@@ -2987,7 +2987,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="2:6">
+    <row r="37" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B37">
         <v>1</v>
       </c>
@@ -3004,7 +3004,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="2:6">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B38">
         <v>1</v>
       </c>
@@ -3021,7 +3021,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="39" spans="2:6">
+    <row r="39" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B39">
         <v>1</v>
       </c>
@@ -3038,7 +3038,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="40" spans="2:6">
+    <row r="40" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B40">
         <v>1</v>
       </c>
@@ -3055,7 +3055,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="2:6">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B42">
         <v>2</v>
       </c>
@@ -3072,7 +3072,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="43" spans="2:6">
+    <row r="43" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B43">
         <v>2</v>
       </c>
@@ -3089,7 +3089,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="2:6">
+    <row r="44" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B44">
         <v>2</v>
       </c>
@@ -3106,7 +3106,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="45" spans="2:6">
+    <row r="45" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B45">
         <v>2</v>
       </c>
@@ -3123,7 +3123,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="46" spans="2:6">
+    <row r="46" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B46">
         <v>2</v>
       </c>
@@ -3140,7 +3140,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="2:6">
+    <row r="47" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B47">
         <v>2</v>
       </c>
@@ -3157,7 +3157,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="2:6">
+    <row r="48" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B48">
         <v>2</v>
       </c>
@@ -3174,7 +3174,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="2:6">
+    <row r="50" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B50">
         <v>2</v>
       </c>
@@ -3191,7 +3191,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="2:6">
+    <row r="51" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B51">
         <v>2</v>
       </c>
@@ -3208,7 +3208,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="52" spans="2:6">
+    <row r="52" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B52">
         <v>2</v>
       </c>
@@ -3225,7 +3225,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="53" spans="2:6">
+    <row r="53" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B53">
         <v>2</v>
       </c>
@@ -3242,7 +3242,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="2:6">
+    <row r="54" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B54">
         <v>2</v>
       </c>
@@ -3259,7 +3259,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="55" spans="2:6">
+    <row r="55" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B55">
         <v>2</v>
       </c>
@@ -3276,7 +3276,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="57" spans="2:6">
+    <row r="57" spans="2:6" ht="17" x14ac:dyDescent="0.2">
       <c r="B57">
         <v>2</v>
       </c>
@@ -3293,7 +3293,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="58" spans="2:6">
+    <row r="58" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B58">
         <v>2</v>
       </c>
@@ -3310,7 +3310,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="2:6">
+    <row r="59" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B59">
         <v>2</v>
       </c>
@@ -3327,7 +3327,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="60" spans="2:6">
+    <row r="60" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B60">
         <v>2</v>
       </c>
@@ -3344,7 +3344,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="61" spans="2:6">
+    <row r="61" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B61">
         <v>2</v>
       </c>
@@ -3361,7 +3361,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="62" spans="2:6">
+    <row r="62" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B62">
         <v>2</v>
       </c>
@@ -3378,7 +3378,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="64" spans="2:6">
+    <row r="64" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B64">
         <v>2</v>
       </c>
@@ -3395,7 +3395,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="65" spans="2:6">
+    <row r="65" spans="2:6" ht="17" x14ac:dyDescent="0.2">
       <c r="B65">
         <v>2</v>
       </c>
@@ -3412,7 +3412,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="66" spans="2:6">
+    <row r="66" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B66">
         <v>2</v>
       </c>
@@ -3429,7 +3429,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="67" spans="2:6">
+    <row r="67" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B67">
         <v>2</v>
       </c>
@@ -3446,7 +3446,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="68" spans="2:6">
+    <row r="68" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B68">
         <v>2</v>
       </c>
@@ -3463,7 +3463,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="69" spans="2:6">
+    <row r="69" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B69">
         <v>2</v>
       </c>
@@ -3480,7 +3480,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="71" spans="2:6">
+    <row r="71" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B71">
         <v>2</v>
       </c>
@@ -3497,7 +3497,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="72" spans="2:6">
+    <row r="72" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B72">
         <v>2</v>
       </c>
@@ -3514,7 +3514,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="2:6">
+    <row r="73" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B73">
         <v>2</v>
       </c>
@@ -3531,7 +3531,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="74" spans="2:6">
+    <row r="74" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B74">
         <v>2</v>
       </c>
@@ -3548,7 +3548,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="75" spans="2:6">
+    <row r="75" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B75">
         <v>2</v>
       </c>
@@ -3565,7 +3565,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="76" spans="2:6">
+    <row r="76" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B76">
         <v>2</v>
       </c>
@@ -3582,7 +3582,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="77" spans="2:6">
+    <row r="77" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B77">
         <v>2</v>
       </c>
@@ -3599,7 +3599,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="78" spans="2:6">
+    <row r="78" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B78">
         <v>2</v>
       </c>
@@ -3616,7 +3616,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="80" spans="2:6">
+    <row r="80" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B80">
         <v>3</v>
       </c>
@@ -3633,7 +3633,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="81" spans="2:6">
+    <row r="81" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B81">
         <v>3</v>
       </c>
@@ -3650,7 +3650,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="82" spans="2:6">
+    <row r="82" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B82">
         <v>3</v>
       </c>
@@ -3667,7 +3667,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="83" spans="2:6">
+    <row r="83" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B83">
         <v>3</v>
       </c>
@@ -3684,7 +3684,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="2:6">
+    <row r="85" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B85">
         <v>3</v>
       </c>
@@ -3701,7 +3701,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="86" spans="2:6">
+    <row r="86" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B86">
         <v>3</v>
       </c>
@@ -3718,7 +3718,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="87" spans="2:6">
+    <row r="87" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B87">
         <v>3</v>
       </c>
@@ -3735,7 +3735,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="88" spans="2:6">
+    <row r="88" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B88">
         <v>3</v>
       </c>
@@ -3752,7 +3752,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="89" spans="2:6">
+    <row r="89" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B89">
         <v>3</v>
       </c>
@@ -3769,7 +3769,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="90" spans="2:6">
+    <row r="90" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B90">
         <v>3</v>
       </c>
@@ -3786,7 +3786,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="91" spans="2:6">
+    <row r="91" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B91">
         <v>3</v>
       </c>
@@ -3803,7 +3803,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="92" spans="2:6">
+    <row r="92" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B92">
         <v>3</v>
       </c>
@@ -3820,7 +3820,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="93" spans="2:6">
+    <row r="93" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B93">
         <v>3</v>
       </c>
@@ -3837,7 +3837,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="94" spans="2:6">
+    <row r="94" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B94">
         <v>3</v>
       </c>
@@ -3854,7 +3854,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="95" spans="2:6">
+    <row r="95" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B95">
         <v>3</v>
       </c>
@@ -3871,9 +3871,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="97" spans="2:5">
+    <row r="97" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B97">
         <v>3</v>
+      </c>
+      <c r="C97" t="s">
+        <v>203</v>
       </c>
       <c r="D97" s="3" t="s">
         <v>87</v>
@@ -3881,10 +3884,16 @@
       <c r="E97" s="2" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="98" spans="2:5">
+      <c r="F97">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="98" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B98">
         <v>3</v>
+      </c>
+      <c r="C98" t="s">
+        <v>203</v>
       </c>
       <c r="D98" s="3" t="s">
         <v>87</v>
@@ -3892,10 +3901,16 @@
       <c r="E98" s="2" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="99" spans="2:5">
+      <c r="F98">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="99" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B99">
         <v>3</v>
+      </c>
+      <c r="C99" t="s">
+        <v>203</v>
       </c>
       <c r="D99" s="3" t="s">
         <v>87</v>
@@ -3903,10 +3918,16 @@
       <c r="E99" s="2" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="100" spans="2:5">
+      <c r="F99">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="100" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B100">
         <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>203</v>
       </c>
       <c r="D100" s="3" t="s">
         <v>87</v>
@@ -3914,10 +3935,16 @@
       <c r="E100" s="2" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="101" spans="2:5">
+      <c r="F100">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="101" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B101">
         <v>3</v>
+      </c>
+      <c r="C101" t="s">
+        <v>203</v>
       </c>
       <c r="D101" s="3" t="s">
         <v>87</v>
@@ -3925,10 +3952,16 @@
       <c r="E101" s="2" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="102" spans="2:5">
+      <c r="F101">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="102" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B102">
         <v>3</v>
+      </c>
+      <c r="C102" t="s">
+        <v>203</v>
       </c>
       <c r="D102" s="3" t="s">
         <v>87</v>
@@ -3936,10 +3969,16 @@
       <c r="E102" s="2" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="103" spans="2:5">
+      <c r="F102">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="103" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B103">
         <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>203</v>
       </c>
       <c r="D103" s="3" t="s">
         <v>87</v>
@@ -3947,10 +3986,16 @@
       <c r="E103" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="104" spans="2:5">
+      <c r="F103">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="104" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B104">
         <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>203</v>
       </c>
       <c r="D104" s="3" t="s">
         <v>87</v>
@@ -3958,10 +4003,16 @@
       <c r="E104" s="2" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="105" spans="2:5">
+      <c r="F104">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="105" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B105">
         <v>3</v>
+      </c>
+      <c r="C105" t="s">
+        <v>203</v>
       </c>
       <c r="D105" s="3" t="s">
         <v>87</v>
@@ -3969,10 +4020,16 @@
       <c r="E105" s="2" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="106" spans="2:5">
+      <c r="F105">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="106" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B106">
         <v>3</v>
+      </c>
+      <c r="C106" t="s">
+        <v>203</v>
       </c>
       <c r="D106" s="3" t="s">
         <v>87</v>
@@ -3980,10 +4037,16 @@
       <c r="E106" s="2" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="108" spans="2:5">
+      <c r="F106">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="108" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B108">
         <v>3</v>
+      </c>
+      <c r="C108" t="s">
+        <v>203</v>
       </c>
       <c r="D108" s="3" t="s">
         <v>98</v>
@@ -3991,10 +4054,16 @@
       <c r="E108" s="2" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="109" spans="2:5">
+      <c r="F108">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="109" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B109">
         <v>3</v>
+      </c>
+      <c r="C109" t="s">
+        <v>203</v>
       </c>
       <c r="D109" s="3" t="s">
         <v>98</v>
@@ -4002,10 +4071,16 @@
       <c r="E109" s="2" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="110" spans="2:5">
+      <c r="F109">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="110" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B110">
         <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>203</v>
       </c>
       <c r="D110" s="3" t="s">
         <v>98</v>
@@ -4013,10 +4088,16 @@
       <c r="E110" s="2" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="111" spans="2:5">
+      <c r="F110">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="111" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B111">
         <v>3</v>
+      </c>
+      <c r="C111" t="s">
+        <v>203</v>
       </c>
       <c r="D111" s="3" t="s">
         <v>98</v>
@@ -4024,10 +4105,16 @@
       <c r="E111" s="2" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="112" spans="2:5">
+      <c r="F111">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="112" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B112">
         <v>3</v>
+      </c>
+      <c r="C112" t="s">
+        <v>203</v>
       </c>
       <c r="D112" s="3" t="s">
         <v>98</v>
@@ -4035,10 +4122,16 @@
       <c r="E112" s="2" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="114" spans="2:5">
+      <c r="F112">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="114" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B114">
         <v>3</v>
+      </c>
+      <c r="C114" t="s">
+        <v>203</v>
       </c>
       <c r="D114" s="3" t="s">
         <v>104</v>
@@ -4046,10 +4139,16 @@
       <c r="E114" s="2" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="115" spans="2:5">
+      <c r="F114">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="115" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B115">
         <v>3</v>
+      </c>
+      <c r="C115" t="s">
+        <v>203</v>
       </c>
       <c r="D115" s="3" t="s">
         <v>104</v>
@@ -4057,10 +4156,16 @@
       <c r="E115" s="2" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="116" spans="2:5">
+      <c r="F115">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="116" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B116">
         <v>3</v>
+      </c>
+      <c r="C116" t="s">
+        <v>203</v>
       </c>
       <c r="D116" s="3" t="s">
         <v>104</v>
@@ -4068,8 +4173,11 @@
       <c r="E116" s="2" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="118" spans="2:5">
+      <c r="F116">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="118" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B118">
         <v>4</v>
       </c>
@@ -4080,7 +4188,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="119" spans="2:5">
+    <row r="119" spans="2:6" ht="17" x14ac:dyDescent="0.2">
       <c r="B119">
         <v>4</v>
       </c>
@@ -4091,7 +4199,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="120" spans="2:5">
+    <row r="120" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B120">
         <v>4</v>
       </c>
@@ -4102,7 +4210,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="121" spans="2:5">
+    <row r="121" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B121">
         <v>4</v>
       </c>
@@ -4113,7 +4221,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="122" spans="2:5">
+    <row r="122" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B122">
         <v>4</v>
       </c>
@@ -4124,7 +4232,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="123" spans="2:5">
+    <row r="123" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B123">
         <v>4</v>
       </c>
@@ -4135,7 +4243,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="125" spans="2:5">
+    <row r="125" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B125">
         <v>4</v>
       </c>
@@ -4146,7 +4254,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="126" spans="2:5">
+    <row r="126" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B126">
         <v>4</v>
       </c>
@@ -4157,7 +4265,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="127" spans="2:5">
+    <row r="127" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B127">
         <v>4</v>
       </c>
@@ -4168,7 +4276,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="128" spans="2:5">
+    <row r="128" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B128">
         <v>4</v>
       </c>
@@ -4179,7 +4287,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="129" spans="2:5">
+    <row r="129" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B129">
         <v>4</v>
       </c>
@@ -4190,7 +4298,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="130" spans="2:5">
+    <row r="130" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B130">
         <v>4</v>
       </c>
@@ -4201,7 +4309,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="131" spans="2:5">
+    <row r="131" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B131">
         <v>4</v>
       </c>
@@ -4212,7 +4320,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="132" spans="2:5">
+    <row r="132" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B132">
         <v>4</v>
       </c>
@@ -4223,7 +4331,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="133" spans="2:5">
+    <row r="133" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B133">
         <v>4</v>
       </c>
@@ -4234,7 +4342,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="134" spans="2:5">
+    <row r="134" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B134">
         <v>4</v>
       </c>
@@ -4245,7 +4353,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="135" spans="2:5">
+    <row r="135" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B135">
         <v>4</v>
       </c>
@@ -4256,7 +4364,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="137" spans="2:5">
+    <row r="137" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B137">
         <v>4</v>
       </c>
@@ -4267,7 +4375,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="138" spans="2:5">
+    <row r="138" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B138">
         <v>4</v>
       </c>
@@ -4278,7 +4386,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="139" spans="2:5">
+    <row r="139" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B139">
         <v>4</v>
       </c>
@@ -4289,7 +4397,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="140" spans="2:5">
+    <row r="140" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B140">
         <v>4</v>
       </c>
@@ -4300,7 +4408,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="142" spans="2:5">
+    <row r="142" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B142">
         <v>4</v>
       </c>
@@ -4311,7 +4419,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="143" spans="2:5">
+    <row r="143" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B143">
         <v>4</v>
       </c>
@@ -4322,7 +4430,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="144" spans="2:5">
+    <row r="144" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B144">
         <v>4</v>
       </c>
@@ -4333,7 +4441,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="145" spans="2:5">
+    <row r="145" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B145">
         <v>4</v>
       </c>
@@ -4344,7 +4452,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="146" spans="2:5">
+    <row r="146" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B146">
         <v>4</v>
       </c>
@@ -4355,7 +4463,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="147" spans="2:5">
+    <row r="147" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B147">
         <v>4</v>
       </c>
@@ -4366,7 +4474,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="148" spans="2:5">
+    <row r="148" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B148">
         <v>4</v>
       </c>
@@ -4377,7 +4485,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="150" spans="2:5">
+    <row r="150" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B150">
         <v>4</v>
       </c>
@@ -4388,7 +4496,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="151" spans="2:5">
+    <row r="151" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B151">
         <v>4</v>
       </c>
@@ -4399,7 +4507,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="152" spans="2:5">
+    <row r="152" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B152">
         <v>4</v>
       </c>
@@ -4410,7 +4518,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="153" spans="2:5">
+    <row r="153" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B153">
         <v>4</v>
       </c>
@@ -4421,7 +4529,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="154" spans="2:5">
+    <row r="154" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B154">
         <v>4</v>
       </c>
@@ -4432,7 +4540,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="155" spans="2:5">
+    <row r="155" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B155">
         <v>4</v>
       </c>
@@ -4443,7 +4551,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="156" spans="2:5">
+    <row r="156" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B156">
         <v>4</v>
       </c>
@@ -4454,7 +4562,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="157" spans="2:5">
+    <row r="157" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B157">
         <v>4</v>
       </c>
@@ -4465,7 +4573,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="158" spans="2:5">
+    <row r="158" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B158">
         <v>4</v>
       </c>
@@ -4476,7 +4584,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="159" spans="2:5">
+    <row r="159" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B159">
         <v>4</v>
       </c>
@@ -4487,7 +4595,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="161" spans="2:5">
+    <row r="161" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B161">
         <v>5</v>
       </c>
@@ -4498,7 +4606,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="162" spans="2:5">
+    <row r="162" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B162">
         <v>5</v>
       </c>
@@ -4509,7 +4617,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="163" spans="2:5">
+    <row r="163" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B163">
         <v>5</v>
       </c>
@@ -4520,7 +4628,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="164" spans="2:5">
+    <row r="164" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B164">
         <v>5</v>
       </c>
@@ -4531,7 +4639,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="165" spans="2:5">
+    <row r="165" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B165">
         <v>5</v>
       </c>
@@ -4542,7 +4650,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="166" spans="2:5">
+    <row r="166" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B166">
         <v>5</v>
       </c>
@@ -4553,7 +4661,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="167" spans="2:5">
+    <row r="167" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B167">
         <v>5</v>
       </c>
@@ -4564,7 +4672,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="169" spans="2:5">
+    <row r="169" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B169">
         <v>5</v>
       </c>
@@ -4575,7 +4683,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="170" spans="2:5">
+    <row r="170" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B170">
         <v>5</v>
       </c>
@@ -4586,7 +4694,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="171" spans="2:5">
+    <row r="171" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B171">
         <v>5</v>
       </c>
@@ -4597,7 +4705,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="172" spans="2:5">
+    <row r="172" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B172">
         <v>5</v>
       </c>
@@ -4608,7 +4716,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="173" spans="2:5">
+    <row r="173" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B173">
         <v>5</v>
       </c>
@@ -4619,7 +4727,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="175" spans="2:5">
+    <row r="175" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B175">
         <v>5</v>
       </c>
@@ -4630,7 +4738,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="176" spans="2:5">
+    <row r="176" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B176">
         <v>5</v>
       </c>
@@ -4641,7 +4749,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="177" spans="2:5">
+    <row r="177" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B177">
         <v>5</v>
       </c>
@@ -4652,7 +4760,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="178" spans="2:5">
+    <row r="178" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B178">
         <v>5</v>
       </c>
@@ -4663,7 +4771,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="179" spans="2:5">
+    <row r="179" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B179">
         <v>5</v>
       </c>
@@ -4674,7 +4782,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="180" spans="2:5">
+    <row r="180" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B180">
         <v>5</v>
       </c>
@@ -4685,7 +4793,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="181" spans="2:5">
+    <row r="181" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B181">
         <v>5</v>
       </c>
@@ -4696,7 +4804,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="182" spans="2:5">
+    <row r="182" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B182">
         <v>5</v>
       </c>
@@ -4707,7 +4815,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="184" spans="2:5">
+    <row r="184" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B184">
         <v>5</v>
       </c>
@@ -4718,7 +4826,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="185" spans="2:5">
+    <row r="185" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B185">
         <v>5</v>
       </c>
@@ -4729,7 +4837,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="186" spans="2:5">
+    <row r="186" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B186">
         <v>5</v>
       </c>
@@ -4740,7 +4848,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="187" spans="2:5">
+    <row r="187" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B187">
         <v>5</v>
       </c>
@@ -4751,7 +4859,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="188" spans="2:5">
+    <row r="188" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B188">
         <v>5</v>
       </c>
@@ -4762,7 +4870,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="189" spans="2:5">
+    <row r="189" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B189">
         <v>5</v>
       </c>
@@ -4773,7 +4881,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="190" spans="2:5">
+    <row r="190" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B190">
         <v>5</v>
       </c>
@@ -4784,7 +4892,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="191" spans="2:5">
+    <row r="191" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B191">
         <v>5</v>
       </c>
@@ -4795,7 +4903,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="193" spans="4:5">
+    <row r="193" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D193" s="6"/>
       <c r="E193" s="7"/>
     </row>

</xml_diff>

<commit_message>
fix: make llm usage flexible by providing different providers to call apis
</commit_message>
<xml_diff>
--- a/Tasks.xlsx
+++ b/Tasks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jacopodonati/Documents/PROGETTI/TRAVELMINDER/ai-travel-planner/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pas02\Nextcloud\Documents\03_Data Science - Uni Stuttgart\06_SoS 2026\04_Software Engineering\Group project 3\ai-travel-planner\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6465E58-F374-294C-99D3-0E516C95C3C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="2940" windowWidth="30440" windowHeight="16320" xr2:uid="{834F46D4-8CFA-4605-9F2C-653FA769D6F4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{834F46D4-8CFA-4605-9F2C-653FA769D6F4}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -763,7 +763,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -844,7 +844,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -862,7 +862,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="de-DE"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1984,7 +1984,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -2301,16 +2301,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67F1D602-D536-4BC9-865A-CD2C06CAE9C2}">
   <dimension ref="B2:M193"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="6.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
-    <col min="4" max="4" width="29.6640625" customWidth="1"/>
-    <col min="5" max="5" width="66.1640625" customWidth="1"/>
-    <col min="6" max="6" width="12.5" customWidth="1"/>
+    <col min="2" max="2" width="6.85546875" customWidth="1"/>
+    <col min="3" max="3" width="22.85546875" customWidth="1"/>
+    <col min="4" max="4" width="29.7109375" customWidth="1"/>
+    <col min="5" max="5" width="66.140625" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" ht="22" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:13" ht="21">
       <c r="B2" s="5" t="s">
         <v>191</v>
       </c>
@@ -2319,7 +2319,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:13">
       <c r="E3" s="4"/>
       <c r="K3" t="s">
         <v>199</v>
@@ -2328,7 +2328,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:13">
       <c r="B4" s="1" t="s">
         <v>188</v>
       </c>
@@ -2360,7 +2360,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:13">
       <c r="B5">
         <v>1</v>
       </c>
@@ -2393,7 +2393,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:13">
       <c r="B6">
         <v>1</v>
       </c>
@@ -2429,7 +2429,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="7" spans="2:13" ht="17" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:13">
       <c r="B7">
         <v>1</v>
       </c>
@@ -2469,7 +2469,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:13">
       <c r="B8">
         <v>1</v>
       </c>
@@ -2509,7 +2509,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:13">
       <c r="B9">
         <v>1</v>
       </c>
@@ -2549,7 +2549,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:13">
       <c r="B10">
         <v>1</v>
       </c>
@@ -2589,7 +2589,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:13">
       <c r="B11">
         <v>1</v>
       </c>
@@ -2613,7 +2613,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:13">
       <c r="B12">
         <v>1</v>
       </c>
@@ -2630,7 +2630,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:13">
       <c r="B14">
         <v>1</v>
       </c>
@@ -2647,7 +2647,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:13">
       <c r="B15">
         <v>1</v>
       </c>
@@ -2664,7 +2664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="2:13" ht="17" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:13">
       <c r="B16">
         <v>1</v>
       </c>
@@ -2681,7 +2681,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:6">
       <c r="B17">
         <v>1</v>
       </c>
@@ -2698,7 +2698,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:6">
       <c r="B18">
         <v>1</v>
       </c>
@@ -2715,7 +2715,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:6">
       <c r="B19">
         <v>1</v>
       </c>
@@ -2732,7 +2732,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:6">
       <c r="B20">
         <v>1</v>
       </c>
@@ -2749,7 +2749,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:6">
       <c r="B22">
         <v>1</v>
       </c>
@@ -2766,7 +2766,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:6">
       <c r="B23">
         <v>1</v>
       </c>
@@ -2783,7 +2783,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:6">
       <c r="B24">
         <v>1</v>
       </c>
@@ -2800,7 +2800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:6">
       <c r="B25">
         <v>1</v>
       </c>
@@ -2817,7 +2817,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:6">
       <c r="B26">
         <v>1</v>
       </c>
@@ -2834,7 +2834,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:6">
       <c r="B27">
         <v>1</v>
       </c>
@@ -2851,7 +2851,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:6">
       <c r="B28">
         <v>1</v>
       </c>
@@ -2868,7 +2868,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:6">
       <c r="B29">
         <v>1</v>
       </c>
@@ -2885,7 +2885,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:6">
       <c r="B30">
         <v>1</v>
       </c>
@@ -2902,7 +2902,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:6">
       <c r="B31">
         <v>1</v>
       </c>
@@ -2919,7 +2919,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:6">
       <c r="B32">
         <v>1</v>
       </c>
@@ -2936,7 +2936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:6">
       <c r="B33">
         <v>1</v>
       </c>
@@ -2953,7 +2953,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:6">
       <c r="B34">
         <v>1</v>
       </c>
@@ -2970,7 +2970,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:6">
       <c r="B36">
         <v>1</v>
       </c>
@@ -2987,7 +2987,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:6">
       <c r="B37">
         <v>1</v>
       </c>
@@ -3004,7 +3004,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:6">
       <c r="B38">
         <v>1</v>
       </c>
@@ -3021,7 +3021,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:6">
       <c r="B39">
         <v>1</v>
       </c>
@@ -3038,7 +3038,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:6">
       <c r="B40">
         <v>1</v>
       </c>
@@ -3055,7 +3055,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:6">
       <c r="B42">
         <v>2</v>
       </c>
@@ -3072,7 +3072,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:6">
       <c r="B43">
         <v>2</v>
       </c>
@@ -3089,7 +3089,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="2:6">
       <c r="B44">
         <v>2</v>
       </c>
@@ -3106,7 +3106,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="45" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="2:6">
       <c r="B45">
         <v>2</v>
       </c>
@@ -3123,7 +3123,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:6">
       <c r="B46">
         <v>2</v>
       </c>
@@ -3140,7 +3140,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="2:6">
       <c r="B47">
         <v>2</v>
       </c>
@@ -3157,7 +3157,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="2:6">
       <c r="B48">
         <v>2</v>
       </c>
@@ -3174,7 +3174,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:6">
       <c r="B50">
         <v>2</v>
       </c>
@@ -3191,7 +3191,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:6">
       <c r="B51">
         <v>2</v>
       </c>
@@ -3208,7 +3208,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:6">
       <c r="B52">
         <v>2</v>
       </c>
@@ -3225,7 +3225,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="2:6">
       <c r="B53">
         <v>2</v>
       </c>
@@ -3242,7 +3242,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:6">
       <c r="B54">
         <v>2</v>
       </c>
@@ -3259,7 +3259,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="55" spans="2:6">
       <c r="B55">
         <v>2</v>
       </c>
@@ -3276,7 +3276,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="57" spans="2:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="57" spans="2:6">
       <c r="B57">
         <v>2</v>
       </c>
@@ -3293,7 +3293,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="58" spans="2:6">
       <c r="B58">
         <v>2</v>
       </c>
@@ -3310,7 +3310,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="59" spans="2:6">
       <c r="B59">
         <v>2</v>
       </c>
@@ -3327,7 +3327,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="60" spans="2:6">
       <c r="B60">
         <v>2</v>
       </c>
@@ -3344,7 +3344,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="61" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="61" spans="2:6">
       <c r="B61">
         <v>2</v>
       </c>
@@ -3361,7 +3361,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="62" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="62" spans="2:6">
       <c r="B62">
         <v>2</v>
       </c>
@@ -3378,7 +3378,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="2:6">
       <c r="B64">
         <v>2</v>
       </c>
@@ -3395,7 +3395,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="65" spans="2:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="65" spans="2:6">
       <c r="B65">
         <v>2</v>
       </c>
@@ -3412,7 +3412,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="66" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="66" spans="2:6">
       <c r="B66">
         <v>2</v>
       </c>
@@ -3429,7 +3429,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="67" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="67" spans="2:6">
       <c r="B67">
         <v>2</v>
       </c>
@@ -3446,7 +3446,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="68" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="68" spans="2:6">
       <c r="B68">
         <v>2</v>
       </c>
@@ -3463,7 +3463,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="69" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="69" spans="2:6">
       <c r="B69">
         <v>2</v>
       </c>
@@ -3480,7 +3480,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="71" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="71" spans="2:6">
       <c r="B71">
         <v>2</v>
       </c>
@@ -3497,7 +3497,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="72" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="72" spans="2:6">
       <c r="B72">
         <v>2</v>
       </c>
@@ -3514,7 +3514,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="73" spans="2:6">
       <c r="B73">
         <v>2</v>
       </c>
@@ -3531,7 +3531,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="74" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="74" spans="2:6">
       <c r="B74">
         <v>2</v>
       </c>
@@ -3548,7 +3548,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="75" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="75" spans="2:6">
       <c r="B75">
         <v>2</v>
       </c>
@@ -3565,7 +3565,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="76" spans="2:6">
       <c r="B76">
         <v>2</v>
       </c>
@@ -3582,7 +3582,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="77" spans="2:6">
       <c r="B77">
         <v>2</v>
       </c>
@@ -3599,7 +3599,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="78" spans="2:6">
       <c r="B78">
         <v>2</v>
       </c>
@@ -3616,7 +3616,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="80" spans="2:6">
       <c r="B80">
         <v>3</v>
       </c>
@@ -3633,7 +3633,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="81" spans="2:6">
       <c r="B81">
         <v>3</v>
       </c>
@@ -3650,7 +3650,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="82" spans="2:6">
       <c r="B82">
         <v>3</v>
       </c>
@@ -3667,7 +3667,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="83" spans="2:6">
       <c r="B83">
         <v>3</v>
       </c>
@@ -3684,7 +3684,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="85" spans="2:6">
       <c r="B85">
         <v>3</v>
       </c>
@@ -3701,7 +3701,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="86" spans="2:6">
       <c r="B86">
         <v>3</v>
       </c>
@@ -3718,7 +3718,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="87" spans="2:6">
       <c r="B87">
         <v>3</v>
       </c>
@@ -3735,7 +3735,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="88" spans="2:6">
       <c r="B88">
         <v>3</v>
       </c>
@@ -3752,7 +3752,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="89" spans="2:6">
       <c r="B89">
         <v>3</v>
       </c>
@@ -3769,7 +3769,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="90" spans="2:6">
       <c r="B90">
         <v>3</v>
       </c>
@@ -3786,7 +3786,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="91" spans="2:6">
       <c r="B91">
         <v>3</v>
       </c>
@@ -3803,7 +3803,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="92" spans="2:6">
       <c r="B92">
         <v>3</v>
       </c>
@@ -3820,7 +3820,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="93" spans="2:6">
       <c r="B93">
         <v>3</v>
       </c>
@@ -3837,7 +3837,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="94" spans="2:6">
       <c r="B94">
         <v>3</v>
       </c>
@@ -3854,7 +3854,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="95" spans="2:6">
       <c r="B95">
         <v>3</v>
       </c>
@@ -3871,7 +3871,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="97" spans="2:6">
       <c r="B97">
         <v>3</v>
       </c>
@@ -3888,7 +3888,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="98" spans="2:6">
       <c r="B98">
         <v>3</v>
       </c>
@@ -3905,7 +3905,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="99" spans="2:6">
       <c r="B99">
         <v>3</v>
       </c>
@@ -3922,7 +3922,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="100" spans="2:6">
       <c r="B100">
         <v>3</v>
       </c>
@@ -3939,7 +3939,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="101" spans="2:6">
       <c r="B101">
         <v>3</v>
       </c>
@@ -3956,7 +3956,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="102" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="102" spans="2:6">
       <c r="B102">
         <v>3</v>
       </c>
@@ -3973,7 +3973,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="103" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="103" spans="2:6">
       <c r="B103">
         <v>3</v>
       </c>
@@ -3990,7 +3990,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="104" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="104" spans="2:6">
       <c r="B104">
         <v>3</v>
       </c>
@@ -4007,7 +4007,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="105" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="105" spans="2:6">
       <c r="B105">
         <v>3</v>
       </c>
@@ -4024,7 +4024,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="106" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="106" spans="2:6">
       <c r="B106">
         <v>3</v>
       </c>
@@ -4041,7 +4041,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="108" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="108" spans="2:6">
       <c r="B108">
         <v>3</v>
       </c>
@@ -4058,7 +4058,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="109" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="109" spans="2:6">
       <c r="B109">
         <v>3</v>
       </c>
@@ -4075,7 +4075,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="110" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="110" spans="2:6">
       <c r="B110">
         <v>3</v>
       </c>
@@ -4092,7 +4092,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="111" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="111" spans="2:6">
       <c r="B111">
         <v>3</v>
       </c>
@@ -4109,7 +4109,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="112" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="112" spans="2:6">
       <c r="B112">
         <v>3</v>
       </c>
@@ -4126,7 +4126,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="114" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="114" spans="2:6">
       <c r="B114">
         <v>3</v>
       </c>
@@ -4143,7 +4143,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="115" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="115" spans="2:6">
       <c r="B115">
         <v>3</v>
       </c>
@@ -4160,7 +4160,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="116" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="116" spans="2:6">
       <c r="B116">
         <v>3</v>
       </c>
@@ -4177,7 +4177,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="118" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="118" spans="2:6">
       <c r="B118">
         <v>4</v>
       </c>
@@ -4188,7 +4188,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="119" spans="2:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="119" spans="2:6">
       <c r="B119">
         <v>4</v>
       </c>
@@ -4199,7 +4199,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="120" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="120" spans="2:6">
       <c r="B120">
         <v>4</v>
       </c>
@@ -4210,7 +4210,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="121" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="121" spans="2:6">
       <c r="B121">
         <v>4</v>
       </c>
@@ -4221,7 +4221,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="122" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="122" spans="2:6">
       <c r="B122">
         <v>4</v>
       </c>
@@ -4232,7 +4232,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="123" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="123" spans="2:6">
       <c r="B123">
         <v>4</v>
       </c>
@@ -4243,7 +4243,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="125" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="125" spans="2:6">
       <c r="B125">
         <v>4</v>
       </c>
@@ -4254,7 +4254,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="126" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="126" spans="2:6">
       <c r="B126">
         <v>4</v>
       </c>
@@ -4265,7 +4265,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="127" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="127" spans="2:6">
       <c r="B127">
         <v>4</v>
       </c>
@@ -4276,7 +4276,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="128" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="128" spans="2:6">
       <c r="B128">
         <v>4</v>
       </c>
@@ -4287,7 +4287,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="129" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="129" spans="2:5">
       <c r="B129">
         <v>4</v>
       </c>
@@ -4298,7 +4298,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="130" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="130" spans="2:5">
       <c r="B130">
         <v>4</v>
       </c>
@@ -4309,7 +4309,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="131" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="131" spans="2:5">
       <c r="B131">
         <v>4</v>
       </c>
@@ -4320,7 +4320,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="132" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="132" spans="2:5">
       <c r="B132">
         <v>4</v>
       </c>
@@ -4331,7 +4331,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="133" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="133" spans="2:5">
       <c r="B133">
         <v>4</v>
       </c>
@@ -4342,7 +4342,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="134" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="134" spans="2:5">
       <c r="B134">
         <v>4</v>
       </c>
@@ -4353,7 +4353,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="135" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="135" spans="2:5">
       <c r="B135">
         <v>4</v>
       </c>
@@ -4364,7 +4364,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="137" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="137" spans="2:5">
       <c r="B137">
         <v>4</v>
       </c>
@@ -4375,7 +4375,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="138" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="138" spans="2:5">
       <c r="B138">
         <v>4</v>
       </c>
@@ -4386,7 +4386,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="139" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="139" spans="2:5">
       <c r="B139">
         <v>4</v>
       </c>
@@ -4397,7 +4397,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="140" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="140" spans="2:5">
       <c r="B140">
         <v>4</v>
       </c>
@@ -4408,7 +4408,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="142" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="142" spans="2:5">
       <c r="B142">
         <v>4</v>
       </c>
@@ -4419,7 +4419,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="143" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="143" spans="2:5">
       <c r="B143">
         <v>4</v>
       </c>
@@ -4430,7 +4430,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="144" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="144" spans="2:5">
       <c r="B144">
         <v>4</v>
       </c>
@@ -4441,7 +4441,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="145" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="145" spans="2:5">
       <c r="B145">
         <v>4</v>
       </c>
@@ -4452,7 +4452,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="146" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="146" spans="2:5">
       <c r="B146">
         <v>4</v>
       </c>
@@ -4463,7 +4463,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="147" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="147" spans="2:5">
       <c r="B147">
         <v>4</v>
       </c>
@@ -4474,7 +4474,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="148" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="148" spans="2:5">
       <c r="B148">
         <v>4</v>
       </c>
@@ -4485,7 +4485,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="150" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="150" spans="2:5">
       <c r="B150">
         <v>4</v>
       </c>
@@ -4496,7 +4496,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="151" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="151" spans="2:5">
       <c r="B151">
         <v>4</v>
       </c>
@@ -4507,7 +4507,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="152" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="152" spans="2:5">
       <c r="B152">
         <v>4</v>
       </c>
@@ -4518,7 +4518,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="153" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="153" spans="2:5">
       <c r="B153">
         <v>4</v>
       </c>
@@ -4529,7 +4529,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="154" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="154" spans="2:5">
       <c r="B154">
         <v>4</v>
       </c>
@@ -4540,7 +4540,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="155" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="155" spans="2:5">
       <c r="B155">
         <v>4</v>
       </c>
@@ -4551,7 +4551,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="156" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="156" spans="2:5">
       <c r="B156">
         <v>4</v>
       </c>
@@ -4562,7 +4562,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="157" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="157" spans="2:5">
       <c r="B157">
         <v>4</v>
       </c>
@@ -4573,7 +4573,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="158" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="158" spans="2:5">
       <c r="B158">
         <v>4</v>
       </c>
@@ -4584,7 +4584,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="159" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="159" spans="2:5">
       <c r="B159">
         <v>4</v>
       </c>
@@ -4595,7 +4595,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="161" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="161" spans="2:5">
       <c r="B161">
         <v>5</v>
       </c>
@@ -4606,7 +4606,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="162" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="162" spans="2:5">
       <c r="B162">
         <v>5</v>
       </c>
@@ -4617,7 +4617,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="163" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="163" spans="2:5">
       <c r="B163">
         <v>5</v>
       </c>
@@ -4628,7 +4628,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="164" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="164" spans="2:5">
       <c r="B164">
         <v>5</v>
       </c>
@@ -4639,7 +4639,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="165" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="165" spans="2:5">
       <c r="B165">
         <v>5</v>
       </c>
@@ -4650,7 +4650,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="166" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="166" spans="2:5">
       <c r="B166">
         <v>5</v>
       </c>
@@ -4661,7 +4661,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="167" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="167" spans="2:5">
       <c r="B167">
         <v>5</v>
       </c>
@@ -4672,7 +4672,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="169" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="169" spans="2:5">
       <c r="B169">
         <v>5</v>
       </c>
@@ -4683,7 +4683,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="170" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="170" spans="2:5">
       <c r="B170">
         <v>5</v>
       </c>
@@ -4694,7 +4694,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="171" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="171" spans="2:5">
       <c r="B171">
         <v>5</v>
       </c>
@@ -4705,7 +4705,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="172" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="172" spans="2:5">
       <c r="B172">
         <v>5</v>
       </c>
@@ -4716,7 +4716,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="173" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="173" spans="2:5">
       <c r="B173">
         <v>5</v>
       </c>
@@ -4727,7 +4727,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="175" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="175" spans="2:5">
       <c r="B175">
         <v>5</v>
       </c>
@@ -4738,7 +4738,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="176" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="176" spans="2:5">
       <c r="B176">
         <v>5</v>
       </c>
@@ -4749,7 +4749,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="177" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="177" spans="2:5">
       <c r="B177">
         <v>5</v>
       </c>
@@ -4760,7 +4760,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="178" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="178" spans="2:5">
       <c r="B178">
         <v>5</v>
       </c>
@@ -4771,7 +4771,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="179" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="179" spans="2:5">
       <c r="B179">
         <v>5</v>
       </c>
@@ -4782,7 +4782,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="180" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="180" spans="2:5">
       <c r="B180">
         <v>5</v>
       </c>
@@ -4793,7 +4793,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="181" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="181" spans="2:5">
       <c r="B181">
         <v>5</v>
       </c>
@@ -4804,7 +4804,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="182" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="182" spans="2:5">
       <c r="B182">
         <v>5</v>
       </c>
@@ -4815,7 +4815,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="184" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="184" spans="2:5">
       <c r="B184">
         <v>5</v>
       </c>
@@ -4826,7 +4826,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="185" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="185" spans="2:5">
       <c r="B185">
         <v>5</v>
       </c>
@@ -4837,7 +4837,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="186" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="186" spans="2:5">
       <c r="B186">
         <v>5</v>
       </c>
@@ -4848,7 +4848,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="187" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="187" spans="2:5">
       <c r="B187">
         <v>5</v>
       </c>
@@ -4859,7 +4859,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="188" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="188" spans="2:5">
       <c r="B188">
         <v>5</v>
       </c>
@@ -4870,7 +4870,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="189" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="189" spans="2:5">
       <c r="B189">
         <v>5</v>
       </c>
@@ -4881,7 +4881,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="190" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="190" spans="2:5">
       <c r="B190">
         <v>5</v>
       </c>
@@ -4892,7 +4892,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="191" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="191" spans="2:5">
       <c r="B191">
         <v>5</v>
       </c>
@@ -4903,7 +4903,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="193" spans="4:5" x14ac:dyDescent="0.2">
+    <row r="193" spans="4:5">
       <c r="D193" s="6"/>
       <c r="E193" s="7"/>
     </row>

</xml_diff>

<commit_message>
feat(results): add surprise, regeneration, and pdf export flows
</commit_message>
<xml_diff>
--- a/Tasks.xlsx
+++ b/Tasks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/exler/VSCode_Projects/ai-travel-planner/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDFE2DF2-5246-1A46-98DB-DE4000986756}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40CBEFF7-254B-CB45-AFB2-C142EC3856A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1240" windowWidth="34200" windowHeight="19660" xr2:uid="{834F46D4-8CFA-4605-9F2C-653FA769D6F4}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21460" xr2:uid="{834F46D4-8CFA-4605-9F2C-653FA769D6F4}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -891,7 +891,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="de-DE" b="1"/>
-              <a:t>Alpha Sprint Burn-down chart (day 4)</a:t>
+              <a:t>Alpha Sprint Burn-down chart (day 5)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1070,10 +1070,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Tabelle1!$L$5:$L$9</c:f>
+              <c:f>Tabelle1!$L$5:$L$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
                   <c:v>165</c:v>
                 </c:pt>
@@ -1088,6 +1088,9 @@
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>43</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>26</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2331,7 +2334,7 @@
         <v>199</v>
       </c>
       <c r="L3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.2">
@@ -2580,19 +2583,19 @@
       </c>
       <c r="J10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="K10">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L10" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="M10" t="str">
+      <c r="L10">
+        <f>IF(H10&gt;$L$3,"",L9-J10)</f>
+        <v>26</v>
+      </c>
+      <c r="M10">
         <f>IF(H10&gt;$L$3,"",L10)</f>
-        <v/>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.2">
@@ -4193,6 +4196,9 @@
       <c r="E118" s="2" t="s">
         <v>109</v>
       </c>
+      <c r="F118">
+        <v>5</v>
+      </c>
     </row>
     <row r="119" spans="2:6" ht="17" x14ac:dyDescent="0.2">
       <c r="B119">
@@ -4204,6 +4210,9 @@
       <c r="E119" s="2" t="s">
         <v>187</v>
       </c>
+      <c r="F119">
+        <v>5</v>
+      </c>
     </row>
     <row r="120" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B120">
@@ -4215,6 +4224,9 @@
       <c r="E120" s="2" t="s">
         <v>110</v>
       </c>
+      <c r="F120">
+        <v>5</v>
+      </c>
     </row>
     <row r="121" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B121">
@@ -4226,6 +4238,9 @@
       <c r="E121" s="2" t="s">
         <v>111</v>
       </c>
+      <c r="F121">
+        <v>5</v>
+      </c>
     </row>
     <row r="122" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B122">
@@ -4237,6 +4252,9 @@
       <c r="E122" s="2" t="s">
         <v>112</v>
       </c>
+      <c r="F122">
+        <v>5</v>
+      </c>
     </row>
     <row r="123" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B123">
@@ -4248,6 +4266,9 @@
       <c r="E123" s="2" t="s">
         <v>113</v>
       </c>
+      <c r="F123">
+        <v>5</v>
+      </c>
     </row>
     <row r="125" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B125">
@@ -4446,6 +4467,9 @@
       <c r="E137" s="2" t="s">
         <v>127</v>
       </c>
+      <c r="F137">
+        <v>5</v>
+      </c>
     </row>
     <row r="138" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B138">
@@ -4457,6 +4481,9 @@
       <c r="E138" s="2" t="s">
         <v>128</v>
       </c>
+      <c r="F138">
+        <v>5</v>
+      </c>
     </row>
     <row r="139" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B139">
@@ -4468,6 +4495,9 @@
       <c r="E139" s="2" t="s">
         <v>129</v>
       </c>
+      <c r="F139">
+        <v>5</v>
+      </c>
     </row>
     <row r="140" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B140">
@@ -4479,6 +4509,9 @@
       <c r="E140" s="2" t="s">
         <v>130</v>
       </c>
+      <c r="F140">
+        <v>5</v>
+      </c>
     </row>
     <row r="142" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B142">
@@ -4739,7 +4772,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="161" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="161" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B161">
         <v>5</v>
       </c>
@@ -4749,8 +4782,11 @@
       <c r="E161" s="2" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="162" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F161">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="162" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B162">
         <v>5</v>
       </c>
@@ -4760,8 +4796,11 @@
       <c r="E162" s="2" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="163" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F162">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="163" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B163">
         <v>5</v>
       </c>
@@ -4771,8 +4810,11 @@
       <c r="E163" s="2" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="164" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F163">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="164" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B164">
         <v>5</v>
       </c>
@@ -4782,8 +4824,11 @@
       <c r="E164" s="2" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="165" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F164">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="165" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B165">
         <v>5</v>
       </c>
@@ -4793,8 +4838,11 @@
       <c r="E165" s="2" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="166" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F165">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="166" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B166">
         <v>5</v>
       </c>
@@ -4804,8 +4852,11 @@
       <c r="E166" s="2" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="167" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F166">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="167" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B167">
         <v>5</v>
       </c>
@@ -4815,8 +4866,11 @@
       <c r="E167" s="2" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="169" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F167">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="169" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B169">
         <v>5</v>
       </c>
@@ -4827,7 +4881,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="170" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="170" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B170">
         <v>5</v>
       </c>
@@ -4838,7 +4892,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="171" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="171" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B171">
         <v>5</v>
       </c>
@@ -4849,7 +4903,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="172" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="172" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B172">
         <v>5</v>
       </c>
@@ -4860,7 +4914,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="173" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="173" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B173">
         <v>5</v>
       </c>
@@ -4871,7 +4925,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="175" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="175" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B175">
         <v>5</v>
       </c>
@@ -4882,7 +4936,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="176" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="176" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B176">
         <v>5</v>
       </c>

</xml_diff>